<commit_message>
fix: repair bridge workbook formulas and enforce dossier export gates
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/BANG_BOC_TACH_CHI_TIET_DAM_SUPER_T_38.2M_KM19.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/BANG_BOC_TACH_CHI_TIET_DAM_SUPER_T_38.2M_KM19.xlsx
@@ -2451,11 +2451,9 @@
       <c r="G6" s="31" t="inlineStr"/>
       <c r="H6" s="30">
         <f>SUM(I7:I9)</f>
-        <v/>
       </c>
       <c r="I6" s="32">
         <f>SUM(I7:I9)</f>
-        <v/>
       </c>
       <c r="J6" s="30" t="inlineStr">
         <is>
@@ -2495,7 +2493,6 @@
       </c>
       <c r="I7" s="36">
         <f>_xlfn.LET(_xlpm.n, D7, _xlpm.L, E7, _xlpm.S, 1.605476985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
@@ -2535,7 +2532,6 @@
       </c>
       <c r="I8" s="40">
         <f>_xlfn.LET(_xlpm.n, D8, _xlpm.L, E8, _xlpm.S, 1.650476985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J8" s="38" t="inlineStr">
         <is>
@@ -2575,7 +2571,6 @@
       </c>
       <c r="I9" s="36">
         <f>_xlfn.LET(_xlpm.n, D9, _xlpm.L, E9, _xlpm.S, 0.639042922, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J9" s="34" t="inlineStr">
         <is>
@@ -2612,11 +2607,9 @@
       <c r="G10" s="31" t="inlineStr"/>
       <c r="H10" s="30">
         <f>SUM(I11:I12)</f>
-        <v/>
       </c>
       <c r="I10" s="32">
         <f>SUM(I11:I12)</f>
-        <v/>
       </c>
       <c r="J10" s="30" t="inlineStr">
         <is>
@@ -2656,7 +2649,6 @@
       </c>
       <c r="I11" s="36">
         <f>_xlfn.LET(_xlpm.n, D11, _xlpm.n * 213.8545432)</f>
-        <v/>
       </c>
       <c r="J11" s="34" t="inlineStr">
         <is>
@@ -2696,7 +2688,6 @@
       </c>
       <c r="I12" s="40">
         <f>_xlfn.LET(_xlpm.n, D12, _xlpm.n * 129.277472874)</f>
-        <v/>
       </c>
       <c r="J12" s="38" t="inlineStr">
         <is>
@@ -2754,11 +2745,9 @@
       <c r="G14" s="31" t="inlineStr"/>
       <c r="H14" s="30">
         <f>SUM(I15:I17)</f>
-        <v/>
       </c>
       <c r="I14" s="32">
         <f>SUM(I15:I17)</f>
-        <v/>
       </c>
       <c r="J14" s="30" t="inlineStr">
         <is>
@@ -2798,7 +2787,6 @@
       </c>
       <c r="I15" s="36">
         <f>_xlfn.LET(_xlpm.n, D15, _xlpm.L, E15, _xlpm.S, 1.603601985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
@@ -2838,7 +2826,6 @@
       </c>
       <c r="I16" s="40">
         <f>_xlfn.LET(_xlpm.n, D16, _xlpm.L, E16, _xlpm.S, 1.648601985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J16" s="38" t="inlineStr">
         <is>
@@ -2878,7 +2865,6 @@
       </c>
       <c r="I17" s="36">
         <f>_xlfn.LET(_xlpm.n, D17, _xlpm.L, E17, _xlpm.S, 0.637167922, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
@@ -2915,11 +2901,9 @@
       <c r="G18" s="31" t="inlineStr"/>
       <c r="H18" s="30">
         <f>SUM(I19:I20)</f>
-        <v/>
       </c>
       <c r="I18" s="32">
         <f>SUM(I19:I20)</f>
-        <v/>
       </c>
       <c r="J18" s="30" t="inlineStr">
         <is>
@@ -2959,7 +2943,6 @@
       </c>
       <c r="I19" s="36">
         <f>_xlfn.LET(_xlpm.n, D19, _xlpm.n * 212.8957932)</f>
-        <v/>
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
@@ -2999,7 +2982,6 @@
       </c>
       <c r="I20" s="40">
         <f>_xlfn.LET(_xlpm.n, D20, _xlpm.n * 129.277472874)</f>
-        <v/>
       </c>
       <c r="J20" s="38" t="inlineStr">
         <is>
@@ -3057,11 +3039,9 @@
       <c r="G22" s="31" t="inlineStr"/>
       <c r="H22" s="30">
         <f>SUM(I23:I25)</f>
-        <v/>
       </c>
       <c r="I22" s="32">
         <f>SUM(I23:I25)</f>
-        <v/>
       </c>
       <c r="J22" s="30" t="inlineStr">
         <is>
@@ -3101,7 +3081,6 @@
       </c>
       <c r="I23" s="36">
         <f>_xlfn.LET(_xlpm.n, D23, _xlpm.L, E23, _xlpm.S, 1.598726985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J23" s="34" t="inlineStr">
         <is>
@@ -3141,7 +3120,6 @@
       </c>
       <c r="I24" s="40">
         <f>_xlfn.LET(_xlpm.n, D24, _xlpm.L, E24, _xlpm.S, 1.643726985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J24" s="38" t="inlineStr">
         <is>
@@ -3181,7 +3159,6 @@
       </c>
       <c r="I25" s="36">
         <f>_xlfn.LET(_xlpm.n, D25, _xlpm.L, E25, _xlpm.S, 0.632292922, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J25" s="34" t="inlineStr">
         <is>
@@ -3218,11 +3195,9 @@
       <c r="G26" s="31" t="inlineStr"/>
       <c r="H26" s="30">
         <f>SUM(I27:I28)</f>
-        <v/>
       </c>
       <c r="I26" s="32">
         <f>SUM(I27:I28)</f>
-        <v/>
       </c>
       <c r="J26" s="30" t="inlineStr">
         <is>
@@ -3262,7 +3237,6 @@
       </c>
       <c r="I27" s="36">
         <f>_xlfn.LET(_xlpm.n, D27, _xlpm.n * 210.4030432)</f>
-        <v/>
       </c>
       <c r="J27" s="34" t="inlineStr">
         <is>
@@ -3302,7 +3276,6 @@
       </c>
       <c r="I28" s="40">
         <f>_xlfn.LET(_xlpm.n, D28, _xlpm.n * 129.277472874)</f>
-        <v/>
       </c>
       <c r="J28" s="38" t="inlineStr">
         <is>
@@ -3360,11 +3333,9 @@
       <c r="G30" s="31" t="inlineStr"/>
       <c r="H30" s="30">
         <f>SUM(I31:I33)</f>
-        <v/>
       </c>
       <c r="I30" s="32">
         <f>SUM(I31:I33)</f>
-        <v/>
       </c>
       <c r="J30" s="30" t="inlineStr">
         <is>
@@ -3404,7 +3375,6 @@
       </c>
       <c r="I31" s="36">
         <f>_xlfn.LET(_xlpm.n, D31, _xlpm.L, E31, _xlpm.S, 1.551101985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J31" s="34" t="inlineStr">
         <is>
@@ -3444,7 +3414,6 @@
       </c>
       <c r="I32" s="40">
         <f>_xlfn.LET(_xlpm.n, D32, _xlpm.L, E32, _xlpm.S, 1.641101985, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J32" s="38" t="inlineStr">
         <is>
@@ -3484,7 +3453,6 @@
       </c>
       <c r="I33" s="36">
         <f>_xlfn.LET(_xlpm.n, D33, _xlpm.L, E33, _xlpm.S, 0.629667922, _xlpm.n * _xlpm.S * _xlpm.L)</f>
-        <v/>
       </c>
       <c r="J33" s="34" t="inlineStr">
         <is>
@@ -3521,11 +3489,9 @@
       <c r="G34" s="31" t="inlineStr"/>
       <c r="H34" s="30">
         <f>SUM(I35:I36)</f>
-        <v/>
       </c>
       <c r="I34" s="32">
         <f>SUM(I35:I36)</f>
-        <v/>
       </c>
       <c r="J34" s="30" t="inlineStr">
         <is>
@@ -3565,7 +3531,6 @@
       </c>
       <c r="I35" s="36">
         <f>_xlfn.LET(_xlpm.n, D35, _xlpm.n * 209.2007932)</f>
-        <v/>
       </c>
       <c r="J35" s="34" t="inlineStr">
         <is>
@@ -3605,7 +3570,6 @@
       </c>
       <c r="I36" s="40">
         <f>_xlfn.LET(_xlpm.n, D36, _xlpm.n * 129.277472874)</f>
-        <v/>
       </c>
       <c r="J36" s="38" t="inlineStr">
         <is>
@@ -3668,13 +3632,13 @@
         <v>1.1</v>
       </c>
       <c r="H38" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D38, _xlpm.m1, 1994.08, _xlpm.n * _xlpm.m1)</f>
         <is>
           <t>LET(n, D39, m1, 1994.08, n * m1)</t>
         </is>
       </c>
       <c r="I38" s="41">
-        <f>_xlfn.LET(_xlpm.n, D39, _xlpm.m1, 1994.08, _xlpm.n * _xlpm.m1)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D38, _xlpm.m1, 1994.08, _xlpm.n * _xlpm.m1)</f>
       </c>
       <c r="J38" s="30" t="inlineStr">
         <is>
@@ -3712,13 +3676,13 @@
       <c r="F39" s="31" t="inlineStr"/>
       <c r="G39" s="31" t="inlineStr"/>
       <c r="H39" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D39, _xlpm.L1, E39, _xlpm.n * _xlpm.L1)</f>
         <is>
           <t>LET(n, D40, L1, E40, n * L1)</t>
         </is>
       </c>
       <c r="I39" s="42">
-        <f>_xlfn.LET(_xlpm.n, D40, _xlpm.L1, E40, _xlpm.n * _xlpm.L1)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D39, _xlpm.L1, E39, _xlpm.n * _xlpm.L1)</f>
       </c>
       <c r="J39" s="30" t="inlineStr">
         <is>
@@ -3760,13 +3724,13 @@
         <v>0.02</v>
       </c>
       <c r="H40" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D40, _xlpm.L, E40, _xlpm.W, F40, _xlpm.t, G40, _xlpm.n * _xlpm.L * _xlpm.W * _xlpm.t * 7850)</f>
         <is>
           <t>LET(n, D41, L, E41, W, F41, t, G41, n*L*W*t*7850)</t>
         </is>
       </c>
       <c r="I40" s="41">
-        <f>_xlfn.LET(_xlpm.n, D41, _xlpm.L, E41, _xlpm.W, F41, _xlpm.t, G41, _xlpm.n * _xlpm.L * _xlpm.W * _xlpm.t * 7850)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D40, _xlpm.L, E40, _xlpm.W, F40, _xlpm.t, G40, _xlpm.n * _xlpm.L * _xlpm.W * _xlpm.t * 7850)</f>
       </c>
       <c r="J40" s="30" t="inlineStr">
         <is>
@@ -3808,7 +3772,6 @@
       </c>
       <c r="I41" s="42">
         <f>_xlfn.LET(_xlpm.bb, 6 * 16, _xlpm.bt, 9 * 32, _xlpm.bb + _xlpm.bt)</f>
-        <v/>
       </c>
       <c r="J41" s="30" t="inlineStr">
         <is>
@@ -3846,13 +3809,13 @@
       <c r="F42" s="31" t="inlineStr"/>
       <c r="G42" s="31" t="inlineStr"/>
       <c r="H42" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D42, _xlpm.L, E42, _xlpm.n * _xlpm.L)</f>
         <is>
           <t>LET(n, D43, L, E43, n * L)</t>
         </is>
       </c>
       <c r="I42" s="42">
-        <f>_xlfn.LET(_xlpm.n, D43, _xlpm.L, E43, _xlpm.n * _xlpm.L)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D42, _xlpm.L, E42, _xlpm.n * _xlpm.L)</f>
       </c>
       <c r="J42" s="30" t="inlineStr">
         <is>
@@ -3890,13 +3853,13 @@
       <c r="F43" s="31" t="inlineStr"/>
       <c r="G43" s="31" t="inlineStr"/>
       <c r="H43" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D43, _xlpm.L, E43, _xlpm.n * _xlpm.L)</f>
         <is>
           <t>LET(n, D44, L, E44, n * L)</t>
         </is>
       </c>
       <c r="I43" s="42">
-        <f>_xlfn.LET(_xlpm.n, D44, _xlpm.L, E44, _xlpm.n * _xlpm.L)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D43, _xlpm.L, E43, _xlpm.n * _xlpm.L)</f>
       </c>
       <c r="J43" s="30" t="inlineStr">
         <is>
@@ -3934,13 +3897,13 @@
       <c r="F44" s="31" t="inlineStr"/>
       <c r="G44" s="31" t="inlineStr"/>
       <c r="H44" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D44, _xlpm.S, E44, _xlpm.n * _xlpm.S)</f>
         <is>
           <t>LET(n, D45, S, E45, n * S)</t>
         </is>
       </c>
       <c r="I44" s="32">
-        <f>_xlfn.LET(_xlpm.n, D45, _xlpm.S, E45, _xlpm.n * _xlpm.S)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D44, _xlpm.S, E44, _xlpm.n * _xlpm.S)</f>
       </c>
       <c r="J44" s="30" t="inlineStr">
         <is>
@@ -3998,11 +3961,9 @@
       <c r="G46" s="31" t="inlineStr"/>
       <c r="H46" s="30">
         <f>10549.56 + 15806.43 + 5253.28 + 46112.49</f>
-        <v/>
       </c>
       <c r="I46" s="41">
         <f>10549.56 + 15806.43 + 5253.28 + 46112.49</f>
-        <v/>
       </c>
       <c r="J46" s="30" t="inlineStr">
         <is>
@@ -4039,11 +4000,9 @@
       <c r="G47" s="31" t="inlineStr"/>
       <c r="H47" s="30">
         <f>15*796.47</f>
-        <v/>
       </c>
       <c r="I47" s="41">
         <f>15*796.47</f>
-        <v/>
       </c>
       <c r="J47" s="30" t="inlineStr">
         <is>
@@ -4075,12 +4034,10 @@
       <c r="F48" s="39" t="inlineStr"/>
       <c r="G48" s="39" t="inlineStr"/>
       <c r="H48" s="38">
-        <f>SUM(I48:I49)</f>
-        <v/>
+        <f>SUM(I46:I47)</f>
       </c>
       <c r="I48" s="43">
-        <f>SUM(I48:I49)</f>
-        <v/>
+        <f>SUM(I46:I47)</f>
       </c>
       <c r="J48" s="38" t="inlineStr">
         <is>
@@ -4112,12 +4069,10 @@
       <c r="F49" s="35" t="inlineStr"/>
       <c r="G49" s="35" t="inlineStr"/>
       <c r="H49" s="34">
-        <f>I50/1000</f>
-        <v/>
+        <f>I48/1000</f>
       </c>
       <c r="I49" s="36">
-        <f>I50/1000</f>
-        <v/>
+        <f>I48/1000</f>
       </c>
       <c r="J49" s="34" t="inlineStr">
         <is>
@@ -4176,13 +4131,13 @@
       <c r="F51" s="31" t="inlineStr"/>
       <c r="G51" s="31" t="inlineStr"/>
       <c r="H51" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D51, _xlpm.v1, E51, _xlpm.n * _xlpm.v1)</f>
         <is>
           <t>LET(n, D53, v1, E53, n * v1)</t>
         </is>
       </c>
       <c r="I51" s="32">
-        <f>_xlfn.LET(_xlpm.n, D53, _xlpm.v1, E53, _xlpm.n * _xlpm.v1)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D51, _xlpm.v1, E51, _xlpm.n * _xlpm.v1)</f>
       </c>
       <c r="J51" s="30" t="inlineStr">
         <is>
@@ -4220,13 +4175,13 @@
       <c r="F52" s="31" t="inlineStr"/>
       <c r="G52" s="31" t="inlineStr"/>
       <c r="H52" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D52, _xlpm.s1, E52, _xlpm.n * _xlpm.s1)</f>
         <is>
           <t>LET(n, D54, s1, E54, n * s1)</t>
         </is>
       </c>
       <c r="I52" s="32">
-        <f>_xlfn.LET(_xlpm.n, D54, _xlpm.s1, E54, _xlpm.n * _xlpm.s1)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D52, _xlpm.s1, E52, _xlpm.n * _xlpm.s1)</f>
       </c>
       <c r="J52" s="30" t="inlineStr">
         <is>
@@ -4264,13 +4219,13 @@
       <c r="F53" s="31" t="inlineStr"/>
       <c r="G53" s="31" t="inlineStr"/>
       <c r="H53" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D53, _xlpm.m1, E53, _xlpm.n * _xlpm.m1)</f>
         <is>
           <t>LET(n, D55, m1, E55, n * m1)</t>
         </is>
       </c>
       <c r="I53" s="41">
-        <f>_xlfn.LET(_xlpm.n, D55, _xlpm.m1, E55, _xlpm.n * _xlpm.m1)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D53, _xlpm.m1, E53, _xlpm.n * _xlpm.m1)</f>
       </c>
       <c r="J53" s="30" t="inlineStr">
         <is>
@@ -4308,13 +4263,13 @@
       <c r="F54" s="31" t="inlineStr"/>
       <c r="G54" s="31" t="inlineStr"/>
       <c r="H54" s="30" t="inlineStr">
+        <f>_xlfn.LET(_xlpm.n, D54, _xlpm.m1, E54, _xlpm.n * _xlpm.m1)</f>
         <is>
           <t>LET(n, D56, m1, E56, n * m1)</t>
         </is>
       </c>
       <c r="I54" s="41">
-        <f>_xlfn.LET(_xlpm.n, D56, _xlpm.m1, E56, _xlpm.n * _xlpm.m1)</f>
-        <v/>
+        <f>_xlfn.LET(_xlpm.n, D54, _xlpm.m1, E54, _xlpm.n * _xlpm.m1)</f>
       </c>
       <c r="J54" s="30" t="inlineStr">
         <is>
@@ -4378,11 +4333,9 @@
       </c>
       <c r="H56" s="30">
         <f>'00_TONG_HOP_SUPER_T'!J7</f>
-        <v/>
       </c>
       <c r="I56" s="32">
         <f>'00_TONG_HOP_SUPER_T'!J7</f>
-        <v/>
       </c>
       <c r="J56" s="30" t="inlineStr">
         <is>
@@ -4419,11 +4372,9 @@
       <c r="G57" s="31" t="inlineStr"/>
       <c r="H57" s="30">
         <f>'00_TONG_HOP_SUPER_T'!J14</f>
-        <v/>
       </c>
       <c r="I57" s="41">
         <f>'00_TONG_HOP_SUPER_T'!J14</f>
-        <v/>
       </c>
       <c r="J57" s="30" t="inlineStr">
         <is>
@@ -4460,11 +4411,9 @@
       <c r="G58" s="31" t="inlineStr"/>
       <c r="H58" s="30">
         <f>'00_TONG_HOP_SUPER_T'!J17</f>
-        <v/>
       </c>
       <c r="I58" s="32">
         <f>'00_TONG_HOP_SUPER_T'!J17</f>
-        <v/>
       </c>
       <c r="J58" s="30" t="inlineStr">
         <is>
@@ -4501,11 +4450,9 @@
       <c r="G59" s="31" t="inlineStr"/>
       <c r="H59" s="30">
         <f>'00_TONG_HOP_SUPER_T'!K7</f>
-        <v/>
       </c>
       <c r="I59" s="32">
         <f>'00_TONG_HOP_SUPER_T'!K7</f>
-        <v/>
       </c>
       <c r="J59" s="30" t="inlineStr">
         <is>
@@ -4542,11 +4489,9 @@
       <c r="G60" s="31" t="inlineStr"/>
       <c r="H60" s="30">
         <f>'00_TONG_HOP_SUPER_T'!K14</f>
-        <v/>
       </c>
       <c r="I60" s="41">
         <f>'00_TONG_HOP_SUPER_T'!K14</f>
-        <v/>
       </c>
       <c r="J60" s="30" t="inlineStr">
         <is>
@@ -4583,11 +4528,9 @@
       <c r="G61" s="31" t="inlineStr"/>
       <c r="H61" s="30">
         <f>'00_TONG_HOP_SUPER_T'!L8</f>
-        <v/>
       </c>
       <c r="I61" s="32">
         <f>'00_TONG_HOP_SUPER_T'!L8</f>
-        <v/>
       </c>
       <c r="J61" s="30" t="inlineStr">
         <is>

</xml_diff>